<commit_message>
added doc_lan variable indicating the language of the document
</commit_message>
<xml_diff>
--- a/data/HMD_Cze_doc.xlsx
+++ b/data/HMD_Cze_doc.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edina\Dropbox\ACLSStudium\FS 2026\Deep Learning\Group project\Topic classification of historical political programs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{38FAAE4F-2FC4-4B00-87AD-1A130F000FBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{547494FD-6409-440D-B1CD-8F9F606385ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{BEE97AB3-B9D8-457F-8808-F81ACD5D184B}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="112">
   <si>
     <t>doc_title</t>
   </si>
@@ -373,6 +373,9 @@
   </si>
   <si>
     <t>Strana Statopravni</t>
+  </si>
+  <si>
+    <t>doc_lan</t>
   </si>
 </sst>
 </file>
@@ -832,1142 +835,1292 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{767B645C-FEF8-4E1A-89F6-27EAF8600765}">
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.54296875" style="15" customWidth="1"/>
-    <col min="2" max="3" width="11.81640625" style="15"/>
-    <col min="4" max="4" width="45.08984375" style="15" customWidth="1"/>
-    <col min="5" max="5" width="10.90625" style="16"/>
-    <col min="6" max="10" width="10.90625" style="15"/>
+    <col min="2" max="2" width="18.54296875" style="15" customWidth="1"/>
+    <col min="3" max="4" width="11.81640625" style="15"/>
+    <col min="5" max="5" width="45.08984375" style="15" customWidth="1"/>
+    <col min="6" max="6" width="10.90625" style="16"/>
+    <col min="7" max="11" width="10.90625" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="5">
+      <c r="C2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="5">
         <v>1911</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="7"/>
-      <c r="G2" s="6"/>
+      <c r="G2" s="7"/>
       <c r="H2" s="6"/>
       <c r="I2" s="6"/>
       <c r="J2" s="6"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
+      <c r="K2" s="6"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="5">
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5">
         <v>1907</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="7"/>
-      <c r="G3" s="6"/>
+      <c r="G3" s="7"/>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
       <c r="J3" s="6"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
+      <c r="K3" s="6"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="C4" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="9">
+      <c r="D4" s="9">
         <v>1899</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="6"/>
+      <c r="G4" s="7"/>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
+      <c r="K4" s="6"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="C5" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="5">
+      <c r="D5" s="5">
         <v>1903</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="6"/>
+      <c r="G5" s="7"/>
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
       <c r="J5" s="6"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
+      <c r="K5" s="6"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="C6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="5">
+      <c r="D6" s="5">
         <v>1897</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="E6" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="7"/>
-      <c r="G6" s="6"/>
+      <c r="G6" s="7"/>
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
       <c r="J6" s="6"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
+      <c r="K6" s="6"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="C7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="9">
+      <c r="D7" s="9">
         <v>1910</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="E7" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="7"/>
-      <c r="G7" s="6"/>
+      <c r="G7" s="7"/>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
       <c r="J7" s="6"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" s="11" t="s">
+      <c r="K7" s="6"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="C8" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="11">
+      <c r="D8" s="11">
         <v>1900</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="E8" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="F8" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="F8" s="11"/>
       <c r="G8" s="11"/>
-      <c r="H8" s="13"/>
+      <c r="H8" s="11"/>
       <c r="I8" s="13"/>
       <c r="J8" s="13"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
+      <c r="K8" s="13"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="C9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="5">
+      <c r="D9" s="5">
         <v>1902</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="E9" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F9" s="7"/>
-      <c r="G9" s="6"/>
+      <c r="G9" s="7"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
       <c r="J9" s="6"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
+      <c r="K9" s="6"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="C10" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="5">
+      <c r="D10" s="5">
         <v>1911</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="E10" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="7"/>
-      <c r="G10" s="6"/>
+      <c r="G10" s="7"/>
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
+      <c r="K10" s="6"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="C11" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="9">
+      <c r="D11" s="9">
         <v>1907</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="E11" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="7"/>
-      <c r="G11" s="6"/>
+      <c r="G11" s="7"/>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
+      <c r="K11" s="6"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="C12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="5">
+      <c r="D12" s="5">
         <v>1899</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="E12" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="F12" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F12" s="7"/>
-      <c r="G12" s="6"/>
+      <c r="G12" s="7"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
+      <c r="K12" s="6"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="5">
+      <c r="D13" s="5">
         <v>1907</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F13" s="7"/>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="7"/>
+      <c r="H13" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="I13" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="I13" s="6"/>
       <c r="J13" s="6"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
+      <c r="K13" s="6"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="C14" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="9">
+      <c r="D14" s="9">
         <v>1911</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="E14" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F14" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G14" s="6"/>
+      <c r="G14" s="7" t="s">
+        <v>42</v>
+      </c>
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
+      <c r="K14" s="6"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="5">
+      <c r="D15" s="5">
         <v>1910</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F15" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G15" s="6"/>
+      <c r="G15" s="7" t="s">
+        <v>42</v>
+      </c>
       <c r="H15" s="6"/>
       <c r="I15" s="6"/>
       <c r="J15" s="6"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
+      <c r="K15" s="6"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="5">
+      <c r="D16" s="5">
         <v>1911</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F16" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G16" s="6"/>
+      <c r="G16" s="7" t="s">
+        <v>42</v>
+      </c>
       <c r="H16" s="6"/>
       <c r="I16" s="6"/>
       <c r="J16" s="6"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17" s="4" t="s">
+      <c r="K16" s="6"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="C17" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="5">
+      <c r="D17" s="5">
         <v>1902</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="F17" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F17" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G17" s="6"/>
+      <c r="G17" s="7" t="s">
+        <v>42</v>
+      </c>
       <c r="H17" s="6"/>
       <c r="I17" s="6"/>
       <c r="J17" s="6"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
+      <c r="K17" s="6"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C18" s="9">
+      <c r="C18" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="9">
         <v>1897</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="E18" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="F18" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="F18" s="7"/>
-      <c r="G18" s="6"/>
+      <c r="G18" s="7"/>
       <c r="H18" s="6"/>
       <c r="I18" s="6"/>
       <c r="J18" s="6"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
+      <c r="K18" s="6"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C19" s="5">
+      <c r="C19" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="5">
         <v>1900</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="F19" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="F19" s="7"/>
-      <c r="G19" s="6"/>
+      <c r="G19" s="7"/>
       <c r="H19" s="6"/>
       <c r="I19" s="6"/>
       <c r="J19" s="6"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A20" s="4" t="s">
+      <c r="K19" s="6"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C20" s="5">
+      <c r="C20" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="5">
         <v>1907</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="E20" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="F20" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="F20" s="7"/>
-      <c r="G20" s="6"/>
+      <c r="G20" s="7"/>
       <c r="H20" s="6"/>
       <c r="I20" s="6"/>
       <c r="J20" s="6"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
+      <c r="K20" s="6"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="5">
+      <c r="D21" s="5">
         <v>1896</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="E21" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="F21" s="7"/>
-      <c r="G21" s="6"/>
+      <c r="G21" s="7"/>
       <c r="H21" s="6"/>
       <c r="I21" s="6"/>
       <c r="J21" s="6"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A22" s="4" t="s">
+      <c r="K21" s="6"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C22" s="5">
+      <c r="C22" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="5">
         <v>1911</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="E22" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="F22" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="F22" s="7"/>
-      <c r="G22" s="6" t="s">
+      <c r="G22" s="7"/>
+      <c r="H22" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="H22" s="6"/>
       <c r="I22" s="6"/>
       <c r="J22" s="6"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A23" s="4" t="s">
+      <c r="K22" s="6"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B23" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C23" s="9">
+      <c r="C23" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="9">
         <v>1897</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="E23" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="F23" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F23" s="7"/>
-      <c r="G23" s="6"/>
+      <c r="G23" s="7"/>
       <c r="H23" s="6"/>
       <c r="I23" s="6"/>
       <c r="J23" s="6"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A24" s="4" t="s">
+      <c r="K23" s="6"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C24" s="5">
+      <c r="C24" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="5">
         <v>1911</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="E24" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="F24" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F24" s="7"/>
-      <c r="G24" s="6"/>
+      <c r="G24" s="7"/>
       <c r="H24" s="6"/>
       <c r="I24" s="6"/>
       <c r="J24" s="6"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25" s="4" t="s">
+      <c r="K24" s="6"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>42</v>
+      </c>
+      <c r="B25" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="C25" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="5">
+      <c r="D25" s="5">
         <v>1911</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="E25" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="F25" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="F25" s="7"/>
-      <c r="G25" s="6"/>
+      <c r="G25" s="7"/>
       <c r="H25" s="6"/>
       <c r="I25" s="6"/>
       <c r="J25" s="6"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A26" s="4" t="s">
+      <c r="K25" s="6"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B26" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C26" s="9">
+      <c r="C26" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" s="9">
         <v>1911</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="E26" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="F26" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="F26" s="7"/>
-      <c r="G26" s="6"/>
+      <c r="G26" s="7"/>
       <c r="H26" s="6"/>
       <c r="I26" s="6"/>
       <c r="J26" s="6"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A27" s="4" t="s">
+      <c r="K26" s="6"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>42</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B27" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C27" s="9">
+      <c r="C27" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" s="9">
         <v>1907</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="E27" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="F27" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="F27" s="7"/>
-      <c r="G27" s="6"/>
+      <c r="G27" s="7"/>
       <c r="H27" s="6"/>
       <c r="I27" s="6"/>
       <c r="J27" s="6"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A28" s="4" t="s">
+      <c r="K27" s="6"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="C28" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C28" s="5">
+      <c r="D28" s="5">
         <v>1898</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="E28" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="F28" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F28" s="7"/>
-      <c r="G28" s="6"/>
+      <c r="G28" s="7"/>
       <c r="H28" s="6"/>
       <c r="I28" s="6"/>
       <c r="J28" s="6"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A29" s="4" t="s">
+      <c r="K28" s="6"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B29" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C29" s="5">
+      <c r="C29" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="5">
         <v>1907</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="E29" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="F29" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F29" s="7"/>
-      <c r="G29" s="6"/>
+      <c r="G29" s="7"/>
       <c r="H29" s="6"/>
       <c r="I29" s="6"/>
       <c r="J29" s="6"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A30" s="4" t="s">
+      <c r="K29" s="6"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>42</v>
+      </c>
+      <c r="B30" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B30" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C30" s="5">
+      <c r="C30" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="5">
         <v>1900</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="E30" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="F30" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="F30" s="7"/>
-      <c r="G30" s="6" t="s">
+      <c r="G30" s="7"/>
+      <c r="H30" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="H30" s="6" t="s">
+      <c r="I30" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="I30" s="6"/>
       <c r="J30" s="6"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A31" s="11" t="s">
+      <c r="K30" s="6"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="B31" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C31" s="11">
+      <c r="C31" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" s="11">
         <v>1897</v>
       </c>
-      <c r="D31" s="11" t="s">
+      <c r="E31" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="E31" s="12" t="s">
+      <c r="F31" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11" t="s">
+      <c r="G31" s="11"/>
+      <c r="H31" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="H31" s="13"/>
       <c r="I31" s="13"/>
       <c r="J31" s="13"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A32" s="4" t="s">
+      <c r="K31" s="13"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>42</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="C32" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C32" s="5">
+      <c r="D32" s="5">
         <v>1874</v>
       </c>
-      <c r="D32" s="8" t="s">
+      <c r="E32" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="F32" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="F32" s="7"/>
-      <c r="G32" s="6"/>
+      <c r="G32" s="7"/>
       <c r="H32" s="6"/>
       <c r="I32" s="6"/>
       <c r="J32" s="6"/>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A33" s="4" t="s">
+      <c r="K32" s="6"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B33" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C33" s="5">
+      <c r="C33" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33" s="5">
         <v>1900</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="E33" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="F33" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="F33" s="7"/>
-      <c r="G33" s="6"/>
+      <c r="G33" s="7"/>
       <c r="H33" s="6"/>
       <c r="I33" s="6"/>
       <c r="J33" s="6"/>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A34" s="4" t="s">
+      <c r="K33" s="6"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>42</v>
+      </c>
+      <c r="B34" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C34" s="9">
+      <c r="C34" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" s="9">
         <v>1911</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="E34" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="E34" s="6" t="s">
+      <c r="F34" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="F34" s="7"/>
-      <c r="G34" s="6"/>
+      <c r="G34" s="7"/>
       <c r="H34" s="6"/>
       <c r="I34" s="6"/>
       <c r="J34" s="6"/>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A35" s="4" t="s">
+      <c r="K34" s="6"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>42</v>
+      </c>
+      <c r="B35" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="B35" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C35" s="5">
+      <c r="C35" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35" s="5">
         <v>1897</v>
       </c>
-      <c r="D35" s="8" t="s">
+      <c r="E35" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="F35" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="F35" s="7"/>
-      <c r="G35" s="6"/>
+      <c r="G35" s="7"/>
       <c r="H35" s="6"/>
       <c r="I35" s="6"/>
       <c r="J35" s="6"/>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A36" s="4" t="s">
+      <c r="K35" s="6"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>42</v>
+      </c>
+      <c r="B36" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B36" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C36" s="5">
+      <c r="C36" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" s="5">
         <v>1907</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="E36" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="F36" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="F36" s="7"/>
-      <c r="G36" s="14" t="s">
+      <c r="G36" s="7"/>
+      <c r="H36" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="H36" s="6"/>
       <c r="I36" s="6"/>
       <c r="J36" s="6"/>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A37" s="5" t="s">
+      <c r="K36" s="6"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>42</v>
+      </c>
+      <c r="B37" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="B37" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C37" s="5">
+      <c r="C37" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" s="5">
         <v>1900</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="E37" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="E37" s="16" t="s">
+      <c r="F37" s="16" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A38" s="5" t="s">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>42</v>
+      </c>
+      <c r="B38" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B38" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C38" s="5">
+      <c r="C38" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" s="5">
         <v>1900</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="E38" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E38" s="16" t="s">
+      <c r="F38" s="16" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A39" s="5" t="s">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B39" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C39" s="5">
+      <c r="C39" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" s="5">
         <v>1897</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="E39" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E39" s="16" t="s">
+      <c r="F39" s="16" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A40" s="4" t="s">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B40" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C40" s="9">
+      <c r="C40" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40" s="9">
         <v>1911</v>
       </c>
-      <c r="D40" s="8" t="s">
+      <c r="E40" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="E40" s="6" t="s">
+      <c r="F40" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F40" s="7"/>
-      <c r="G40" s="6"/>
+      <c r="G40" s="7"/>
       <c r="H40" s="6"/>
       <c r="I40" s="6"/>
       <c r="J40" s="6"/>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A41" s="4" t="s">
+      <c r="K40" s="6"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>42</v>
+      </c>
+      <c r="B41" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B41" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C41" s="5">
+      <c r="C41" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" s="5">
         <v>1907</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="E41" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="E41" s="6" t="s">
+      <c r="F41" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F41" s="7"/>
-      <c r="G41" s="7" t="s">
+      <c r="G41" s="7"/>
+      <c r="H41" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="H41" s="6" t="s">
+      <c r="I41" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="I41" s="6"/>
       <c r="J41" s="6"/>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A42" s="4" t="s">
+      <c r="K41" s="6"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>42</v>
+      </c>
+      <c r="B42" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B42" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C42" s="5">
+      <c r="C42" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D42" s="5">
         <v>1911</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="E42" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="E42" s="6" t="s">
+      <c r="F42" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F42" s="7"/>
-      <c r="G42" s="6" t="s">
+      <c r="G42" s="7"/>
+      <c r="H42" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="H42" s="14" t="s">
+      <c r="I42" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="I42" s="6"/>
       <c r="J42" s="6"/>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A43" s="4" t="s">
+      <c r="K42" s="6"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B43" s="8" t="s">
+      <c r="C43" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C43" s="9">
+      <c r="D43" s="9">
         <v>1905</v>
       </c>
-      <c r="D43" s="8" t="s">
+      <c r="E43" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="E43" s="14" t="s">
+      <c r="F43" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="F43" s="7"/>
-      <c r="G43" s="6"/>
+      <c r="G43" s="7"/>
       <c r="H43" s="6"/>
       <c r="I43" s="6"/>
       <c r="J43" s="6"/>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A44" s="4" t="s">
+      <c r="K43" s="6"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>42</v>
+      </c>
+      <c r="B44" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B44" s="8" t="s">
+      <c r="C44" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C44" s="9">
+      <c r="D44" s="9">
         <v>1905</v>
       </c>
-      <c r="D44" s="8" t="s">
+      <c r="E44" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="E44" s="14" t="s">
+      <c r="F44" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="F44" s="7"/>
-      <c r="G44" s="6"/>
+      <c r="G44" s="7"/>
       <c r="H44" s="6"/>
       <c r="I44" s="6"/>
       <c r="J44" s="6"/>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A45" s="4" t="s">
+      <c r="K44" s="6"/>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>42</v>
+      </c>
+      <c r="B45" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="B45" s="8" t="s">
+      <c r="C45" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C45" s="5">
+      <c r="D45" s="5">
         <v>1907</v>
       </c>
-      <c r="D45" s="5" t="s">
+      <c r="E45" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="E45" s="6" t="s">
+      <c r="F45" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="F45" s="7"/>
-      <c r="G45" s="6"/>
+      <c r="G45" s="7"/>
       <c r="H45" s="6"/>
       <c r="I45" s="6"/>
       <c r="J45" s="6"/>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A46" s="4" t="s">
+      <c r="K45" s="6"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>42</v>
+      </c>
+      <c r="B46" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="C46" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C46" s="5">
+      <c r="D46" s="5">
         <v>1898</v>
       </c>
-      <c r="D46" s="5" t="s">
+      <c r="E46" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="E46" s="6" t="s">
+      <c r="F46" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F46" s="7"/>
-      <c r="G46" s="6"/>
+      <c r="G46" s="7"/>
       <c r="H46" s="6"/>
       <c r="I46" s="6"/>
       <c r="J46" s="6"/>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A47" s="4" t="s">
+      <c r="K46" s="6"/>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>42</v>
+      </c>
+      <c r="B47" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="B47" s="8" t="s">
+      <c r="C47" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C47" s="9">
+      <c r="D47" s="9">
         <v>1906</v>
       </c>
-      <c r="D47" s="8" t="s">
+      <c r="E47" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="E47" s="6" t="s">
+      <c r="F47" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F47" s="7"/>
-      <c r="G47" s="6"/>
+      <c r="G47" s="7"/>
       <c r="H47" s="6"/>
       <c r="I47" s="6"/>
       <c r="J47" s="6"/>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A48" s="4" t="s">
+      <c r="K47" s="6"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>42</v>
+      </c>
+      <c r="B48" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="B48" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C48" s="5">
+      <c r="C48" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D48" s="5">
         <v>1907</v>
       </c>
-      <c r="D48" s="5" t="s">
+      <c r="E48" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="E48" s="6" t="s">
+      <c r="F48" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F48" s="7"/>
-      <c r="G48" s="6"/>
+      <c r="G48" s="7"/>
       <c r="H48" s="6"/>
       <c r="I48" s="6"/>
       <c r="J48" s="6"/>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A49" s="4" t="s">
+      <c r="K48" s="6"/>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>42</v>
+      </c>
+      <c r="B49" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B49" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C49" s="5">
+      <c r="C49" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D49" s="5">
         <v>1900</v>
       </c>
-      <c r="D49" s="5" t="s">
+      <c r="E49" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="E49" s="6" t="s">
+      <c r="F49" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F49" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G49" s="6"/>
+      <c r="G49" s="7" t="s">
+        <v>42</v>
+      </c>
       <c r="H49" s="6"/>
       <c r="I49" s="6"/>
       <c r="J49" s="6"/>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A50" s="11" t="s">
+      <c r="K49" s="6"/>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>42</v>
+      </c>
+      <c r="B50" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="B50" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C50" s="11">
+      <c r="C50" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D50" s="11">
         <v>1907</v>
       </c>
-      <c r="D50" s="11" t="s">
+      <c r="E50" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="E50" s="12" t="s">
+      <c r="F50" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="F50" s="11"/>
       <c r="G50" s="11"/>
-      <c r="H50" s="13"/>
+      <c r="H50" s="11"/>
       <c r="I50" s="13"/>
       <c r="J50" s="13"/>
+      <c r="K50" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>